<commit_message>
Sync Excel tracker from markdown files
Generator now parses tracker/*.md for Owner, Status, Evidence, and
Notes fields. Criterion 1.4 populated from gate1 markdown updates.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PCCT_Qualification_Tracker.xlsx
+++ b/PCCT_Qualification_Tracker.xlsx
@@ -923,16 +923,28 @@
           <t>Protocol review + DICOM header</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr"/>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Murali</t>
+        </is>
+      </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>https://elucidbio.sharepoint.com/:w:/r/Technology/Documents/IP/PCCT/PT142_combined_analysis_COMPLETE_FINAL_v1.0.docx?d=w0fe5c7e3207c4790930cac6308e7bde7&amp;csf=1&amp;web=1&amp;e=mQv35o</t>
+        </is>
+      </c>
       <c r="H8" s="4" t="inlineStr"/>
       <c r="I8" s="4" t="inlineStr"/>
-      <c r="J8" s="4" t="inlineStr"/>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Kernel family influences local vessel segment and patient level plaque characterization. Recon settings shoud be standardized for subsequent evaluations especially reproducibility and bias-agreement analyses</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:J8"/>

</xml_diff>